<commit_message>
Phi3 - plain rag output commit
</commit_message>
<xml_diff>
--- a/results/comparison_CoTRAG/CoTRAG_costs.xlsx
+++ b/results/comparison_CoTRAG/CoTRAG_costs.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,13 +472,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>22.93916487693787</v>
+        <v>5.506356477737427</v>
       </c>
       <c r="B2" t="n">
-        <v>157.1875</v>
+        <v>2176.3671875</v>
       </c>
       <c r="C2" t="n">
-        <v>18.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -487,12 +487,1728 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.615044116973877</v>
+        <v>0.472334623336792</v>
       </c>
       <c r="G2" t="n">
-        <v>22.32411813735962</v>
+        <v>5.034018278121948</v>
       </c>
       <c r="H2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>5.391723871231079</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C3" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.277754545211792</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5.113965749740601</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>6.454650163650513</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C4" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.279834508895874</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6.17481255531311</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>7.11798882484436</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.2473671436309814</v>
+      </c>
+      <c r="G5" t="n">
+        <v>6.870619058609009</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>7.432021379470825</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C6" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.2458760738372803</v>
+      </c>
+      <c r="G6" t="n">
+        <v>7.186143159866333</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>9.358683347702026</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C7" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.2452392578125</v>
+      </c>
+      <c r="G7" t="n">
+        <v>9.113441467285156</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6.755396842956543</v>
+      </c>
+      <c r="B8" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C8" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.2460243701934814</v>
+      </c>
+      <c r="G8" t="n">
+        <v>6.509369373321533</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>3.476279497146606</v>
+      </c>
+      <c r="B9" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C9" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.2452657222747803</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3.231011390686035</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>4.163097143173218</v>
+      </c>
+      <c r="B10" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C10" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.2583446502685547</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3.904749870300293</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>3.557737112045288</v>
+      </c>
+      <c r="B11" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C11" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.2449972629547119</v>
+      </c>
+      <c r="G11" t="n">
+        <v>3.312737226486206</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>8.980536937713623</v>
+      </c>
+      <c r="B12" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C12" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.2452139854431152</v>
+      </c>
+      <c r="G12" t="n">
+        <v>8.735320091247559</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>9.844990015029907</v>
+      </c>
+      <c r="B13" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C13" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.2472150325775146</v>
+      </c>
+      <c r="G13" t="n">
+        <v>9.597772121429443</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>4.318399667739868</v>
+      </c>
+      <c r="B14" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C14" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.2449526786804199</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.073444843292236</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>8.271855592727661</v>
+      </c>
+      <c r="B15" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.2441065311431885</v>
+      </c>
+      <c r="G15" t="n">
+        <v>8.027746438980103</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>7.83225679397583</v>
+      </c>
+      <c r="B16" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C16" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.2469477653503418</v>
+      </c>
+      <c r="G16" t="n">
+        <v>7.58530592918396</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>4.580297708511353</v>
+      </c>
+      <c r="B17" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C17" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.244257926940918</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4.336037397384644</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>4.840617179870605</v>
+      </c>
+      <c r="B18" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C18" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.2607929706573486</v>
+      </c>
+      <c r="G18" t="n">
+        <v>4.579821586608887</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>5.174953699111938</v>
+      </c>
+      <c r="B19" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C19" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.2432565689086914</v>
+      </c>
+      <c r="G19" t="n">
+        <v>4.931694984436035</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>231.5381226539612</v>
+      </c>
+      <c r="B20" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C20" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.2423772811889648</v>
+      </c>
+      <c r="G20" t="n">
+        <v>231.2957429885864</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>8.126924276351929</v>
+      </c>
+      <c r="B21" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C21" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1.636052131652832</v>
+      </c>
+      <c r="G21" t="n">
+        <v>6.490869522094727</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>3.520207643508911</v>
+      </c>
+      <c r="B22" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C22" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.2365930080413818</v>
+      </c>
+      <c r="G22" t="n">
+        <v>3.283612012863159</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>10.42373871803284</v>
+      </c>
+      <c r="B23" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C23" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.2375402450561523</v>
+      </c>
+      <c r="G23" t="n">
+        <v>10.18619561195374</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>3.1822829246521</v>
+      </c>
+      <c r="B24" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C24" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.2383480072021484</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2.943931579589844</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>7.874937772750854</v>
+      </c>
+      <c r="B25" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C25" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.2387781143188477</v>
+      </c>
+      <c r="G25" t="n">
+        <v>7.636156797409058</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>9.572970390319824</v>
+      </c>
+      <c r="B26" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C26" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.23722243309021</v>
+      </c>
+      <c r="G26" t="n">
+        <v>9.335745573043823</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>3.249281167984009</v>
+      </c>
+      <c r="B27" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C27" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.2406730651855469</v>
+      </c>
+      <c r="G27" t="n">
+        <v>3.008605480194092</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>5.17281699180603</v>
+      </c>
+      <c r="B28" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C28" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.2384819984436035</v>
+      </c>
+      <c r="G28" t="n">
+        <v>4.934332609176636</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>8.999074220657349</v>
+      </c>
+      <c r="B29" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C29" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.2375671863555908</v>
+      </c>
+      <c r="G29" t="n">
+        <v>8.761504173278809</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>3.136008262634277</v>
+      </c>
+      <c r="B30" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C30" t="n">
+        <v>12</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.236060619354248</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2.899945020675659</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>5.740626096725464</v>
+      </c>
+      <c r="B31" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C31" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.237215518951416</v>
+      </c>
+      <c r="G31" t="n">
+        <v>5.503407955169678</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>5.233722448348999</v>
+      </c>
+      <c r="B32" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C32" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.2383832931518555</v>
+      </c>
+      <c r="G32" t="n">
+        <v>4.995336532592773</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>6.56594181060791</v>
+      </c>
+      <c r="B33" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C33" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.2395989894866943</v>
+      </c>
+      <c r="G33" t="n">
+        <v>6.326339960098267</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>9.785745143890381</v>
+      </c>
+      <c r="B34" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C34" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.2371160984039307</v>
+      </c>
+      <c r="G34" t="n">
+        <v>9.54862642288208</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>4.402201652526855</v>
+      </c>
+      <c r="B35" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C35" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.2389931678771973</v>
+      </c>
+      <c r="G35" t="n">
+        <v>4.163206100463867</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>5.792757034301758</v>
+      </c>
+      <c r="B36" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C36" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.2378437519073486</v>
+      </c>
+      <c r="G36" t="n">
+        <v>5.554910659790039</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>6.811272859573364</v>
+      </c>
+      <c r="B37" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C37" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.2391352653503418</v>
+      </c>
+      <c r="G37" t="n">
+        <v>6.57213568687439</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>4.682608842849731</v>
+      </c>
+      <c r="B38" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C38" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.2404549121856689</v>
+      </c>
+      <c r="G38" t="n">
+        <v>4.442151069641113</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>3.459343671798706</v>
+      </c>
+      <c r="B39" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C39" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.2389004230499268</v>
+      </c>
+      <c r="G39" t="n">
+        <v>3.220440864562988</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>9.884209871292114</v>
+      </c>
+      <c r="B40" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C40" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.2403895854949951</v>
+      </c>
+      <c r="G40" t="n">
+        <v>9.64381742477417</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>10.142653465271</v>
+      </c>
+      <c r="B41" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C41" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.2388386726379395</v>
+      </c>
+      <c r="G41" t="n">
+        <v>9.903812170028687</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>5.213563919067383</v>
+      </c>
+      <c r="B42" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C42" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.2396395206451416</v>
+      </c>
+      <c r="G42" t="n">
+        <v>4.973921775817871</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>4.287548780441284</v>
+      </c>
+      <c r="B43" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C43" t="n">
+        <v>10</v>
+      </c>
+      <c r="D43" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.2362575531005859</v>
+      </c>
+      <c r="G43" t="n">
+        <v>4.051287651062012</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>5.324556112289429</v>
+      </c>
+      <c r="B44" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C44" t="n">
+        <v>11</v>
+      </c>
+      <c r="D44" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.2365083694458008</v>
+      </c>
+      <c r="G44" t="n">
+        <v>5.088045358657837</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>10.67091035842896</v>
+      </c>
+      <c r="B45" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C45" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="D45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.2387313842773438</v>
+      </c>
+      <c r="G45" t="n">
+        <v>10.43217658996582</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>2.861963748931885</v>
+      </c>
+      <c r="B46" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C46" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="D46" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.2375876903533936</v>
+      </c>
+      <c r="G46" t="n">
+        <v>2.624373435974121</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>8.596731185913086</v>
+      </c>
+      <c r="B47" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C47" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="D47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.2380437850952148</v>
+      </c>
+      <c r="G47" t="n">
+        <v>8.358685493469238</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>3.813446760177612</v>
+      </c>
+      <c r="B48" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C48" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="D48" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.2374413013458252</v>
+      </c>
+      <c r="G48" t="n">
+        <v>3.576002836227417</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>6.449628591537476</v>
+      </c>
+      <c r="B49" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C49" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.2375915050506592</v>
+      </c>
+      <c r="G49" t="n">
+        <v>6.212034940719604</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>5.463531732559204</v>
+      </c>
+      <c r="B50" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C50" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="D50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.2367475032806396</v>
+      </c>
+      <c r="G50" t="n">
+        <v>5.226781606674194</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>3.40658974647522</v>
+      </c>
+      <c r="B51" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C51" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="D51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.2362701892852783</v>
+      </c>
+      <c r="G51" t="n">
+        <v>3.17031717300415</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>11.85815119743347</v>
+      </c>
+      <c r="B52" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C52" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="D52" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.2386424541473389</v>
+      </c>
+      <c r="G52" t="n">
+        <v>11.61950540542603</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>3.478484392166138</v>
+      </c>
+      <c r="B53" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C53" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.2374942302703857</v>
+      </c>
+      <c r="G53" t="n">
+        <v>3.240987062454224</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>7.407093524932861</v>
+      </c>
+      <c r="B54" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C54" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="D54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.2358105182647705</v>
+      </c>
+      <c r="G54" t="n">
+        <v>7.171280384063721</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>4.445119619369507</v>
+      </c>
+      <c r="B55" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C55" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.2368981838226318</v>
+      </c>
+      <c r="G55" t="n">
+        <v>4.208219051361084</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>3.863778352737427</v>
+      </c>
+      <c r="B56" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C56" t="n">
+        <v>8</v>
+      </c>
+      <c r="D56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.5134825706481934</v>
+      </c>
+      <c r="G56" t="n">
+        <v>3.350293874740601</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>7.234395980834961</v>
+      </c>
+      <c r="B57" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C57" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.2551999092102051</v>
+      </c>
+      <c r="G57" t="n">
+        <v>6.979194164276123</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>8.294326543807983</v>
+      </c>
+      <c r="B58" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C58" t="n">
+        <v>9</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.2374889850616455</v>
+      </c>
+      <c r="G58" t="n">
+        <v>8.056835412979126</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>3.73823356628418</v>
+      </c>
+      <c r="B59" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C59" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="D59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.2376019954681396</v>
+      </c>
+      <c r="G59" t="n">
+        <v>3.500629186630249</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>6.832760095596313</v>
+      </c>
+      <c r="B60" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C60" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="D60" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.239220142364502</v>
+      </c>
+      <c r="G60" t="n">
+        <v>6.593537569046021</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>2.330227136611938</v>
+      </c>
+      <c r="B61" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C61" t="n">
+        <v>9</v>
+      </c>
+      <c r="D61" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.2374305725097656</v>
+      </c>
+      <c r="G61" t="n">
+        <v>2.092794418334961</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>4.245165109634399</v>
+      </c>
+      <c r="B62" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C62" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.2385215759277344</v>
+      </c>
+      <c r="G62" t="n">
+        <v>4.006641149520874</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>3.199214935302734</v>
+      </c>
+      <c r="B63" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C63" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D63" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.237755298614502</v>
+      </c>
+      <c r="G63" t="n">
+        <v>2.961457490921021</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>238.8339817523956</v>
+      </c>
+      <c r="B64" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C64" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="D64" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.2362930774688721</v>
+      </c>
+      <c r="G64" t="n">
+        <v>238.5976860523224</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>6.41077446937561</v>
+      </c>
+      <c r="B65" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C65" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="D65" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>1.177547454833984</v>
+      </c>
+      <c r="G65" t="n">
+        <v>5.233224153518677</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>9.622566223144531</v>
+      </c>
+      <c r="B66" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C66" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="D66" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0.2380890846252441</v>
+      </c>
+      <c r="G66" t="n">
+        <v>9.384474277496338</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>2.955914735794067</v>
+      </c>
+      <c r="B67" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C67" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="D67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0.2381103038787842</v>
+      </c>
+      <c r="G67" t="n">
+        <v>2.717801809310913</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>7.663787126541138</v>
+      </c>
+      <c r="B68" t="n">
+        <v>2176.3671875</v>
+      </c>
+      <c r="C68" t="n">
+        <v>10</v>
+      </c>
+      <c r="D68" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0.2768197059631348</v>
+      </c>
+      <c r="G68" t="n">
+        <v>7.386964559555054</v>
+      </c>
+      <c r="H68" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>